<commit_message>
Fixed Statistics page and plots
</commit_message>
<xml_diff>
--- a/LST_duties_2025.xlsx
+++ b/LST_duties_2025.xlsx
@@ -103,7 +103,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="497">
   <si>
     <t xml:space="preserve">PBS</t>
   </si>
@@ -687,7 +687,7 @@
     <t xml:space="preserve">5.1.1</t>
   </si>
   <si>
-    <t xml:space="preserve">IT container HW</t>
+    <t xml:space="preserve">IT container</t>
   </si>
   <si>
     <t xml:space="preserve">onsite team</t>
@@ -696,25 +696,25 @@
     <t xml:space="preserve">5.1.2</t>
   </si>
   <si>
-    <t xml:space="preserve">IT in CC container HW</t>
+    <t xml:space="preserve">IT in CC container</t>
   </si>
   <si>
     <t xml:space="preserve">5.1.3</t>
   </si>
   <si>
-    <t xml:space="preserve">Webcams HW</t>
+    <t xml:space="preserve">Webcams</t>
   </si>
   <si>
     <t xml:space="preserve">5.1.4</t>
   </si>
   <si>
-    <t xml:space="preserve">Weather station HW</t>
+    <t xml:space="preserve">Weather station</t>
   </si>
   <si>
     <t xml:space="preserve">5.1.5</t>
   </si>
   <si>
-    <t xml:space="preserve">Network LST HW</t>
+    <t xml:space="preserve">Network LST</t>
   </si>
   <si>
     <t xml:space="preserve">5.2</t>
@@ -810,7 +810,7 @@
     <t xml:space="preserve">5.3.3</t>
   </si>
   <si>
-    <t xml:space="preserve">ECC HW</t>
+    <t xml:space="preserve">ECC</t>
   </si>
   <si>
     <t xml:space="preserve">Armand Fiasson (2023) </t>
@@ -846,7 +846,7 @@
     <t xml:space="preserve">5.3.7</t>
   </si>
   <si>
-    <t xml:space="preserve">TIB/UCTS HW</t>
+    <t xml:space="preserve">TIB/UCTS</t>
   </si>
   <si>
     <t xml:space="preserve">Alejandro Perez (2019)</t>
@@ -1050,25 +1050,19 @@
     <t xml:space="preserve">6.1.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Webcams SW</t>
-  </si>
-  <si>
     <t xml:space="preserve">Jarred</t>
   </si>
   <si>
     <t xml:space="preserve">6.1.2</t>
   </si>
   <si>
-    <t xml:space="preserve">Weather Station SW</t>
-  </si>
-  <si>
     <t xml:space="preserve">Alice</t>
   </si>
   <si>
     <t xml:space="preserve">6.1.3</t>
   </si>
   <si>
-    <t xml:space="preserve">Webservers SW</t>
+    <t xml:space="preserve">Webservers</t>
   </si>
   <si>
     <t xml:space="preserve">Michiko, Vitalii</t>
@@ -1077,7 +1071,7 @@
     <t xml:space="preserve">6.1.4</t>
   </si>
   <si>
-    <t xml:space="preserve">ACS Bridges SW</t>
+    <t xml:space="preserve">ACS Bridges</t>
   </si>
   <si>
     <t xml:space="preserve">Jean-Luc, Grzegorz</t>
@@ -1086,7 +1080,7 @@
     <t xml:space="preserve">6.1.5</t>
   </si>
   <si>
-    <t xml:space="preserve">MOS SFW</t>
+    <t xml:space="preserve">MOS</t>
   </si>
   <si>
     <t xml:space="preserve">Jean-Luc</t>
@@ -1095,21 +1089,18 @@
     <t xml:space="preserve">6.1.6</t>
   </si>
   <si>
-    <t xml:space="preserve">Data broker SW</t>
+    <t xml:space="preserve">Data broker</t>
   </si>
   <si>
     <t xml:space="preserve">6.1.7</t>
   </si>
   <si>
-    <t xml:space="preserve">Data broker visualisation SW</t>
+    <t xml:space="preserve">Data broker visualisation</t>
   </si>
   <si>
     <t xml:space="preserve">6.1.8</t>
   </si>
   <si>
-    <t xml:space="preserve">Structure Monitoring SW</t>
-  </si>
-  <si>
     <t xml:space="preserve">6.1.9</t>
   </si>
   <si>
@@ -1128,7 +1119,7 @@
     <t xml:space="preserve">6.2.1</t>
   </si>
   <si>
-    <t xml:space="preserve">TCU &amp; eGui SW</t>
+    <t xml:space="preserve">TCU &amp; eGui</t>
   </si>
   <si>
     <t xml:space="preserve">Ievgen, Vitalii</t>
@@ -1158,16 +1149,10 @@
     <t xml:space="preserve">6.3.2</t>
   </si>
   <si>
-    <t xml:space="preserve">ECC SW</t>
-  </si>
-  <si>
     <t xml:space="preserve">Armand Fiasson, Jean-Luc Panazol</t>
   </si>
   <si>
     <t xml:space="preserve">6.3.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIB/UCTS SW</t>
   </si>
   <si>
     <t xml:space="preserve">Alejandro Perez, María Molina</t>
@@ -5196,7 +5181,7 @@
       </c>
       <c r="C111" s="35"/>
       <c r="D111" s="36" t="s">
-        <v>313</v>
+        <v>197</v>
       </c>
       <c r="E111" s="19" t="s">
         <v>15</v>
@@ -5214,17 +5199,17 @@
       <c r="I111" s="20"/>
       <c r="J111" s="21"/>
       <c r="K111" s="21" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A112" s="16"/>
       <c r="B112" s="15" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C112" s="35"/>
       <c r="D112" s="36" t="s">
-        <v>316</v>
+        <v>199</v>
       </c>
       <c r="E112" s="19" t="s">
         <v>15</v>
@@ -5242,17 +5227,17 @@
       <c r="I112" s="20"/>
       <c r="J112" s="21"/>
       <c r="K112" s="21" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A113" s="16"/>
       <c r="B113" s="15" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C113" s="35"/>
       <c r="D113" s="36" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="E113" s="19" t="s">
         <v>15</v>
@@ -5270,17 +5255,17 @@
       <c r="I113" s="20"/>
       <c r="J113" s="21"/>
       <c r="K113" s="21" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A114" s="16"/>
       <c r="B114" s="15" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C114" s="35"/>
       <c r="D114" s="36" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="E114" s="19" t="s">
         <v>15</v>
@@ -5298,17 +5283,17 @@
       <c r="I114" s="20"/>
       <c r="J114" s="21"/>
       <c r="K114" s="21" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A115" s="16"/>
       <c r="B115" s="15" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C115" s="35"/>
       <c r="D115" s="36" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="E115" s="19" t="s">
         <v>15</v>
@@ -5326,17 +5311,17 @@
       <c r="I115" s="20"/>
       <c r="J115" s="21"/>
       <c r="K115" s="21" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A116" s="16"/>
       <c r="B116" s="15" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C116" s="35"/>
       <c r="D116" s="36" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E116" s="19" t="s">
         <v>15</v>
@@ -5353,17 +5338,17 @@
       <c r="I116" s="20"/>
       <c r="J116" s="21"/>
       <c r="K116" s="21" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A117" s="16"/>
       <c r="B117" s="15" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C117" s="35"/>
       <c r="D117" s="36" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E117" s="19" t="s">
         <v>15</v>
@@ -5380,17 +5365,17 @@
       <c r="I117" s="20"/>
       <c r="J117" s="21"/>
       <c r="K117" s="21" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A118" s="16"/>
       <c r="B118" s="15" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C118" s="35"/>
       <c r="D118" s="36" t="s">
-        <v>332</v>
+        <v>292</v>
       </c>
       <c r="E118" s="19" t="s">
         <v>15</v>
@@ -5412,11 +5397,11 @@
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A119" s="16"/>
       <c r="B119" s="15" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="C119" s="35"/>
       <c r="D119" s="36" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="E119" s="19" t="s">
         <v>15</v>
@@ -5434,16 +5419,16 @@
       <c r="I119" s="20"/>
       <c r="J119" s="21"/>
       <c r="K119" s="21" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A120" s="15" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="B120" s="16"/>
       <c r="C120" s="17" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="D120" s="18"/>
       <c r="E120" s="19"/>
@@ -5460,11 +5445,11 @@
     <row r="121" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A121" s="16"/>
       <c r="B121" s="15" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C121" s="35"/>
       <c r="D121" s="36" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E121" s="19" t="s">
         <v>15</v>
@@ -5482,17 +5467,17 @@
       <c r="I121" s="20"/>
       <c r="J121" s="21"/>
       <c r="K121" s="21" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A122" s="16"/>
       <c r="B122" s="15" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C122" s="35"/>
       <c r="D122" s="36" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="E122" s="19" t="s">
         <v>15</v>
@@ -5510,12 +5495,12 @@
       <c r="I122" s="20"/>
       <c r="J122" s="21"/>
       <c r="K122" s="21" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A123" s="15" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="B123" s="16"/>
       <c r="C123" s="17" t="s">
@@ -5536,11 +5521,11 @@
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A124" s="16"/>
       <c r="B124" s="15" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="C124" s="35"/>
       <c r="D124" s="36" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="E124" s="19" t="s">
         <v>15</v>
@@ -5558,17 +5543,17 @@
       <c r="I124" s="20"/>
       <c r="J124" s="21"/>
       <c r="K124" s="21" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A125" s="16"/>
       <c r="B125" s="15" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="C125" s="35"/>
       <c r="D125" s="36" t="s">
-        <v>349</v>
+        <v>233</v>
       </c>
       <c r="E125" s="19" t="s">
         <v>15</v>
@@ -5586,17 +5571,17 @@
       <c r="I125" s="20"/>
       <c r="J125" s="21"/>
       <c r="K125" s="21" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A126" s="16"/>
       <c r="B126" s="15" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="C126" s="35"/>
       <c r="D126" s="36" t="s">
-        <v>352</v>
+        <v>245</v>
       </c>
       <c r="E126" s="19" t="s">
         <v>15</v>
@@ -5614,17 +5599,17 @@
       <c r="I126" s="20"/>
       <c r="J126" s="21"/>
       <c r="K126" s="21" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A127" s="16"/>
       <c r="B127" s="15" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="C127" s="35"/>
       <c r="D127" s="36" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="E127" s="19" t="s">
         <v>15</v>
@@ -5642,17 +5627,17 @@
       <c r="I127" s="20"/>
       <c r="J127" s="21"/>
       <c r="K127" s="21" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A128" s="16"/>
       <c r="B128" s="15" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="C128" s="35"/>
       <c r="D128" s="36" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="E128" s="19" t="s">
         <v>15</v>
@@ -5670,17 +5655,17 @@
       <c r="I128" s="20"/>
       <c r="J128" s="21"/>
       <c r="K128" s="21" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A129" s="16"/>
       <c r="B129" s="15" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="C129" s="35"/>
       <c r="D129" s="36" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="E129" s="19" t="s">
         <v>15</v>
@@ -5698,17 +5683,17 @@
       <c r="I129" s="20"/>
       <c r="J129" s="21"/>
       <c r="K129" s="21" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A130" s="16"/>
       <c r="B130" s="15" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="C130" s="35"/>
       <c r="D130" s="36" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="E130" s="19" t="s">
         <v>15</v>
@@ -5726,17 +5711,17 @@
       <c r="I130" s="20"/>
       <c r="J130" s="21"/>
       <c r="K130" s="21" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A131" s="16"/>
       <c r="B131" s="15" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="C131" s="35"/>
       <c r="D131" s="36" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="E131" s="19" t="s">
         <v>15</v>
@@ -5752,16 +5737,16 @@
         <v>4</v>
       </c>
       <c r="I131" s="20" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="J131" s="21"/>
       <c r="K131" s="21" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="1" collapsed="false">
       <c r="A132" s="15" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="B132" s="16"/>
       <c r="C132" s="17" t="s">
@@ -5782,11 +5767,11 @@
     <row r="133" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A133" s="16"/>
       <c r="B133" s="15" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="C133" s="35"/>
       <c r="D133" s="36" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="E133" s="19" t="s">
         <v>15</v>
@@ -5804,17 +5789,17 @@
       <c r="I133" s="20"/>
       <c r="J133" s="21"/>
       <c r="K133" s="21" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A134" s="16"/>
       <c r="B134" s="15" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="C134" s="35"/>
       <c r="D134" s="36" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="E134" s="19" t="s">
         <v>15</v>
@@ -5832,12 +5817,12 @@
       <c r="I134" s="20"/>
       <c r="J134" s="21"/>
       <c r="K134" s="21" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A135" s="15" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="B135" s="16"/>
       <c r="C135" s="17" t="s">
@@ -5858,11 +5843,11 @@
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A136" s="16"/>
       <c r="B136" s="15" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="C136" s="35"/>
       <c r="D136" s="36" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="E136" s="19" t="s">
         <v>15</v>
@@ -5880,17 +5865,17 @@
       <c r="I136" s="20"/>
       <c r="J136" s="21"/>
       <c r="K136" s="21" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A137" s="16"/>
       <c r="B137" s="15" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="C137" s="35"/>
       <c r="D137" s="36" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="E137" s="19" t="s">
         <v>15</v>
@@ -5908,17 +5893,17 @@
       <c r="I137" s="20"/>
       <c r="J137" s="21"/>
       <c r="K137" s="21" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A138" s="16"/>
       <c r="B138" s="15" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="C138" s="35"/>
       <c r="D138" s="36" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E138" s="19" t="s">
         <v>15</v>
@@ -5936,12 +5921,12 @@
       <c r="I138" s="20"/>
       <c r="J138" s="21"/>
       <c r="K138" s="21" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A139" s="15" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B139" s="16"/>
       <c r="C139" s="17" t="s">
@@ -5962,11 +5947,11 @@
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A140" s="16"/>
       <c r="B140" s="15" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="C140" s="35"/>
       <c r="D140" s="36" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="E140" s="19" t="s">
         <v>15</v>
@@ -5984,17 +5969,17 @@
       <c r="I140" s="20"/>
       <c r="J140" s="21"/>
       <c r="K140" s="21" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A141" s="16"/>
       <c r="B141" s="15" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="C141" s="35"/>
       <c r="D141" s="36" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="E141" s="19" t="s">
         <v>15</v>
@@ -6012,17 +5997,17 @@
       <c r="I141" s="20"/>
       <c r="J141" s="21"/>
       <c r="K141" s="21" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A142" s="16"/>
       <c r="B142" s="15" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="C142" s="35"/>
       <c r="D142" s="36" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="E142" s="19" t="s">
         <v>15</v>
@@ -6040,17 +6025,17 @@
       <c r="I142" s="20"/>
       <c r="J142" s="21"/>
       <c r="K142" s="21" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A143" s="16"/>
       <c r="B143" s="15" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="C143" s="35"/>
       <c r="D143" s="36" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="E143" s="19" t="s">
         <v>15</v>
@@ -6072,11 +6057,11 @@
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A144" s="16"/>
       <c r="B144" s="15" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="C144" s="35"/>
       <c r="D144" s="36" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="E144" s="19" t="s">
         <v>15</v>
@@ -6094,16 +6079,16 @@
       <c r="I144" s="20"/>
       <c r="J144" s="21"/>
       <c r="K144" s="21" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A145" s="15" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="B145" s="16"/>
       <c r="C145" s="17" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="D145" s="18"/>
       <c r="E145" s="19"/>
@@ -6120,11 +6105,11 @@
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A146" s="16"/>
       <c r="B146" s="15" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="C146" s="35"/>
       <c r="D146" s="36" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="E146" s="19" t="s">
         <v>15</v>
@@ -6140,21 +6125,21 @@
         <v>0</v>
       </c>
       <c r="I146" s="20" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="J146" s="21"/>
       <c r="K146" s="21" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A147" s="16"/>
       <c r="B147" s="15" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="C147" s="39"/>
       <c r="D147" s="40" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="E147" s="19" t="s">
         <v>15</v>
@@ -6170,21 +6155,21 @@
         <v>0</v>
       </c>
       <c r="I147" s="20" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="J147" s="21"/>
       <c r="K147" s="21" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A148" s="16"/>
       <c r="B148" s="42" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="C148" s="39"/>
       <c r="D148" s="40" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="E148" s="19" t="s">
         <v>15</v>
@@ -6200,21 +6185,21 @@
         <v>0</v>
       </c>
       <c r="I148" s="20" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="J148" s="21"/>
       <c r="K148" s="43" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A149" s="16"/>
       <c r="B149" s="42" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="C149" s="39"/>
       <c r="D149" s="40" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="E149" s="19" t="s">
         <v>15</v>
@@ -6230,21 +6215,21 @@
         <v>0</v>
       </c>
       <c r="I149" s="20" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="J149" s="21"/>
       <c r="K149" s="21" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A150" s="16"/>
       <c r="B150" s="42" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="C150" s="39"/>
       <c r="D150" s="40" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="E150" s="19" t="s">
         <v>15</v>
@@ -6260,21 +6245,21 @@
         <v>0</v>
       </c>
       <c r="I150" s="20" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="J150" s="21"/>
       <c r="K150" s="21" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A151" s="16"/>
       <c r="B151" s="42" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="C151" s="39"/>
       <c r="D151" s="40" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="E151" s="19" t="s">
         <v>15</v>
@@ -6290,21 +6275,21 @@
         <v>0</v>
       </c>
       <c r="I151" s="20" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="J151" s="21"/>
       <c r="K151" s="21" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A152" s="16"/>
       <c r="B152" s="42" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="C152" s="39"/>
       <c r="D152" s="40" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="E152" s="19" t="s">
         <v>15</v>
@@ -6320,21 +6305,21 @@
         <v>0</v>
       </c>
       <c r="I152" s="20" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="J152" s="21"/>
       <c r="K152" s="21" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A153" s="16"/>
       <c r="B153" s="42" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="C153" s="39"/>
       <c r="D153" s="40" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
       <c r="E153" s="19" t="s">
         <v>15</v>
@@ -6350,21 +6335,21 @@
         <v>0</v>
       </c>
       <c r="I153" s="20" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="J153" s="21"/>
       <c r="K153" s="21" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A154" s="16"/>
       <c r="B154" s="42" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="C154" s="39"/>
       <c r="D154" s="40" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="E154" s="19" t="s">
         <v>15</v>
@@ -6380,20 +6365,20 @@
         <v>0</v>
       </c>
       <c r="I154" s="20" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="J154" s="21"/>
       <c r="K154" s="21" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A155" s="15" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="B155" s="16"/>
       <c r="C155" s="17" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="D155" s="18"/>
       <c r="E155" s="19"/>
@@ -6410,11 +6395,11 @@
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A156" s="16"/>
       <c r="B156" s="15" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="C156" s="35"/>
       <c r="D156" s="36" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
       <c r="E156" s="19" t="s">
         <v>15</v>
@@ -6432,17 +6417,17 @@
       <c r="I156" s="20"/>
       <c r="J156" s="21"/>
       <c r="K156" s="21" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A157" s="16"/>
       <c r="B157" s="15" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="C157" s="35"/>
       <c r="D157" s="36" t="s">
-        <v>444</v>
+        <v>439</v>
       </c>
       <c r="E157" s="19" t="s">
         <v>15</v>
@@ -6459,18 +6444,18 @@
       </c>
       <c r="I157" s="20"/>
       <c r="J157" s="21" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="K157" s="21" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="31" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="B158" s="32" t="s">
-        <v>448</v>
+        <v>443</v>
       </c>
       <c r="C158" s="37"/>
       <c r="D158" s="37"/>
@@ -6493,11 +6478,11 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A159" s="15" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="B159" s="16"/>
       <c r="C159" s="17" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
       <c r="D159" s="18"/>
       <c r="E159" s="19"/>
@@ -6511,11 +6496,11 @@
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A160" s="16"/>
       <c r="B160" s="15" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="C160" s="17"/>
       <c r="D160" s="18" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="E160" s="19" t="s">
         <v>15</v>
@@ -6533,17 +6518,17 @@
       <c r="I160" s="20"/>
       <c r="J160" s="21"/>
       <c r="K160" s="21" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A161" s="16"/>
       <c r="B161" s="15" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
       <c r="C161" s="17"/>
       <c r="D161" s="18" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
       <c r="E161" s="19" t="s">
         <v>15</v>
@@ -6561,17 +6546,17 @@
       <c r="I161" s="20"/>
       <c r="J161" s="21"/>
       <c r="K161" s="21" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A162" s="16"/>
       <c r="B162" s="15" t="s">
-        <v>457</v>
+        <v>452</v>
       </c>
       <c r="C162" s="17"/>
       <c r="D162" s="18" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="E162" s="19" t="s">
         <v>15</v>
@@ -6589,17 +6574,17 @@
       <c r="I162" s="20"/>
       <c r="J162" s="21"/>
       <c r="K162" s="21" t="s">
-        <v>459</v>
+        <v>454</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A163" s="16"/>
       <c r="B163" s="15" t="s">
-        <v>460</v>
+        <v>455</v>
       </c>
       <c r="C163" s="17"/>
       <c r="D163" s="18" t="s">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="E163" s="19" t="s">
         <v>15</v>
@@ -6621,11 +6606,11 @@
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
       <c r="A164" s="16"/>
       <c r="B164" s="15" t="s">
-        <v>462</v>
+        <v>457</v>
       </c>
       <c r="C164" s="17"/>
       <c r="D164" s="18" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="E164" s="19" t="s">
         <v>15</v>
@@ -6643,16 +6628,16 @@
       <c r="I164" s="20"/>
       <c r="J164" s="21"/>
       <c r="K164" s="21" t="s">
-        <v>464</v>
+        <v>459</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A165" s="15" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B165" s="16"/>
       <c r="C165" s="17" t="s">
-        <v>466</v>
+        <v>461</v>
       </c>
       <c r="D165" s="18"/>
       <c r="E165" s="19" t="s">
@@ -6667,10 +6652,10 @@
     </row>
     <row r="166" customFormat="false" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="31" t="s">
-        <v>467</v>
+        <v>462</v>
       </c>
       <c r="B166" s="32" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
       <c r="C166" s="37"/>
       <c r="D166" s="37"/>
@@ -6693,11 +6678,11 @@
     </row>
     <row r="167" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="15" t="s">
-        <v>469</v>
+        <v>464</v>
       </c>
       <c r="B167" s="16"/>
       <c r="C167" s="45" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="D167" s="18"/>
       <c r="E167" s="19" t="s">
@@ -6715,15 +6700,15 @@
       </c>
       <c r="I167" s="20"/>
       <c r="J167" s="21" t="s">
-        <v>471</v>
+        <v>466</v>
       </c>
       <c r="K167" s="21" t="s">
-        <v>472</v>
+        <v>467</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="15" t="s">
-        <v>473</v>
+        <v>468</v>
       </c>
       <c r="B168" s="16"/>
       <c r="C168" s="45" t="s">
@@ -6745,7 +6730,7 @@
     </row>
     <row r="169" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="15" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="B169" s="16"/>
       <c r="C169" s="45" t="s">
@@ -6765,15 +6750,15 @@
       </c>
       <c r="I169" s="20"/>
       <c r="J169" s="21" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="K169" s="21" t="s">
-        <v>476</v>
+        <v>471</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="15" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="B170" s="16"/>
       <c r="C170" s="45" t="s">
@@ -6793,13 +6778,13 @@
       </c>
       <c r="I170" s="20"/>
       <c r="J170" s="21" t="s">
-        <v>478</v>
+        <v>473</v>
       </c>
       <c r="K170" s="21"/>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="15" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="B171" s="16"/>
       <c r="C171" s="45" t="s">
@@ -6821,11 +6806,11 @@
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="15" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="B172" s="16"/>
       <c r="C172" s="45" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="D172" s="18"/>
       <c r="E172" s="19" t="s">
@@ -6843,10 +6828,10 @@
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="31" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="B173" s="32" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
       <c r="C173" s="37"/>
       <c r="D173" s="37"/>
@@ -6869,11 +6854,11 @@
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="15" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="B174" s="16"/>
       <c r="C174" s="17" t="s">
-        <v>485</v>
+        <v>480</v>
       </c>
       <c r="D174" s="18"/>
       <c r="E174" s="19" t="s">
@@ -6892,16 +6877,16 @@
       <c r="I174" s="20"/>
       <c r="J174" s="21"/>
       <c r="K174" s="21" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="15" t="s">
-        <v>487</v>
+        <v>482</v>
       </c>
       <c r="B175" s="16"/>
       <c r="C175" s="17" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
       <c r="D175" s="18"/>
       <c r="E175" s="19" t="s">
@@ -6920,16 +6905,16 @@
       <c r="I175" s="20"/>
       <c r="J175" s="21"/>
       <c r="K175" s="21" t="s">
-        <v>489</v>
+        <v>484</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="15" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="B176" s="16"/>
       <c r="C176" s="17" t="s">
-        <v>491</v>
+        <v>486</v>
       </c>
       <c r="D176" s="18"/>
       <c r="E176" s="19" t="s">
@@ -6948,16 +6933,16 @@
       <c r="I176" s="20"/>
       <c r="J176" s="21"/>
       <c r="K176" s="21" t="s">
-        <v>492</v>
+        <v>487</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="15" t="s">
-        <v>493</v>
+        <v>488</v>
       </c>
       <c r="B177" s="16"/>
       <c r="C177" s="17" t="s">
-        <v>494</v>
+        <v>489</v>
       </c>
       <c r="D177" s="18"/>
       <c r="E177" s="19" t="s">
@@ -6976,15 +6961,15 @@
       <c r="I177" s="20"/>
       <c r="J177" s="21"/>
       <c r="K177" s="21" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
       <c r="L177" s="43" t="s">
-        <v>496</v>
+        <v>491</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="15" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
       <c r="B178" s="16"/>
       <c r="C178" s="17" t="s">
@@ -7007,16 +6992,16 @@
       <c r="I178" s="20"/>
       <c r="J178" s="21"/>
       <c r="K178" s="21" t="s">
-        <v>498</v>
+        <v>493</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="15" t="s">
-        <v>499</v>
+        <v>494</v>
       </c>
       <c r="B179" s="16"/>
       <c r="C179" s="17" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="D179" s="18"/>
       <c r="E179" s="19" t="s">
@@ -7035,12 +7020,12 @@
       <c r="I179" s="20"/>
       <c r="J179" s="21"/>
       <c r="K179" s="21" t="s">
-        <v>500</v>
+        <v>495</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="46" t="s">
-        <v>501</v>
+        <v>496</v>
       </c>
       <c r="B180" s="47"/>
       <c r="C180" s="35"/>

</xml_diff>